<commit_message>
Stok listesi güncellendi (2026-09-28 21:38)
</commit_message>
<xml_diff>
--- a/stok-listesi.xlsx
+++ b/stok-listesi.xlsx
@@ -46,46 +46,46 @@
     <t>0,63*1340 R</t>
   </si>
   <si>
+    <t>1004</t>
+  </si>
+  <si>
+    <t>0,65*1410 R</t>
+  </si>
+  <si>
+    <t>0,65*1445 R</t>
+  </si>
+  <si>
+    <t>1001</t>
+  </si>
+  <si>
+    <t>0,7*935 R</t>
+  </si>
+  <si>
+    <t>0,7*1140 R</t>
+  </si>
+  <si>
+    <t>0,75*981 R</t>
+  </si>
+  <si>
+    <t>1001 - (1312)</t>
+  </si>
+  <si>
+    <t>0,8*1100 R</t>
+  </si>
+  <si>
+    <t>0,85*1000 R</t>
+  </si>
+  <si>
+    <t>0,9*1170 R</t>
+  </si>
+  <si>
+    <t>0,9*1445 R</t>
+  </si>
+  <si>
+    <t>1,5*1200*2400</t>
+  </si>
+  <si>
     <t>A2</t>
-  </si>
-  <si>
-    <t>0,65*1410 R</t>
-  </si>
-  <si>
-    <t>0,65*1445 R</t>
-  </si>
-  <si>
-    <t>1001</t>
-  </si>
-  <si>
-    <t>0,7*935 R</t>
-  </si>
-  <si>
-    <t>0,7*1140 R</t>
-  </si>
-  <si>
-    <t>1004</t>
-  </si>
-  <si>
-    <t>0,75*981 R</t>
-  </si>
-  <si>
-    <t>1001 - (1312)</t>
-  </si>
-  <si>
-    <t>0,8*1100 R</t>
-  </si>
-  <si>
-    <t>0,85*1000 R</t>
-  </si>
-  <si>
-    <t>0,9*1170 R</t>
-  </si>
-  <si>
-    <t>0,9*1445 R</t>
-  </si>
-  <si>
-    <t>1,5*1200*2400</t>
   </si>
   <si>
     <t>1,7*1020 R</t>
@@ -815,10 +815,10 @@
         <v>5</v>
       </c>
       <c r="B11" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="C11" s="7" t="s">
         <v>17</v>
-      </c>
-      <c r="C11" s="7" t="s">
-        <v>18</v>
       </c>
       <c r="D11" s="8">
         <v>17540</v>
@@ -829,10 +829,10 @@
         <v>5</v>
       </c>
       <c r="B12" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="C12" s="7" t="s">
         <v>17</v>
-      </c>
-      <c r="C12" s="7" t="s">
-        <v>18</v>
       </c>
       <c r="D12" s="8">
         <v>17730</v>
@@ -843,10 +843,10 @@
         <v>5</v>
       </c>
       <c r="B13" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="C13" s="4" t="s">
         <v>19</v>
-      </c>
-      <c r="C13" s="4" t="s">
-        <v>20</v>
       </c>
       <c r="D13" s="5">
         <v>10370</v>
@@ -860,7 +860,7 @@
         <v>14</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D14" s="5">
         <v>9590</v>
@@ -874,7 +874,7 @@
         <v>6</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D15" s="5">
         <v>11200</v>
@@ -888,7 +888,7 @@
         <v>9</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D16" s="5">
         <v>16570</v>
@@ -899,10 +899,10 @@
         <v>5</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D17" s="5">
         <v>3760</v>
@@ -913,7 +913,7 @@
         <v>5</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>11</v>
+        <v>24</v>
       </c>
       <c r="C18" s="4" t="s">
         <v>25</v>
@@ -927,7 +927,7 @@
         <v>5</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>11</v>
+        <v>24</v>
       </c>
       <c r="C19" s="4" t="s">
         <v>26</v>
@@ -1005,7 +1005,7 @@
         <v>28</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>11</v>
+        <v>24</v>
       </c>
       <c r="C25" s="4" t="s">
         <v>35</v>
@@ -1019,7 +1019,7 @@
         <v>28</v>
       </c>
       <c r="B26" s="4" t="s">
-        <v>11</v>
+        <v>24</v>
       </c>
       <c r="C26" s="4" t="s">
         <v>36</v>
@@ -1069,7 +1069,7 @@
         <v>38</v>
       </c>
       <c r="B30" s="4" t="s">
-        <v>11</v>
+        <v>24</v>
       </c>
       <c r="C30" s="4" t="s">
         <v>41</v>
@@ -1181,7 +1181,7 @@
         <v>38</v>
       </c>
       <c r="B38" s="4" t="s">
-        <v>11</v>
+        <v>24</v>
       </c>
       <c r="C38" s="4" t="s">
         <v>53</v>
@@ -1223,7 +1223,7 @@
         <v>38</v>
       </c>
       <c r="B41" s="4" t="s">
-        <v>11</v>
+        <v>24</v>
       </c>
       <c r="C41" s="4" t="s">
         <v>57</v>

</xml_diff>

<commit_message>
Stok listesi güncellendi (2026-09-28 21:42)
</commit_message>
<xml_diff>
--- a/stok-listesi.xlsx
+++ b/stok-listesi.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="154" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="151" uniqueCount="72">
   <si>
     <t>G A L V A N İ Z L İ   Ü R Ü N L E R</t>
   </si>
@@ -667,7 +667,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D53"/>
+  <dimension ref="A1:D52"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -723,7 +723,7 @@
         <v>8</v>
       </c>
       <c r="D4" s="5">
-        <v>17792</v>
+        <v>18730</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
@@ -731,13 +731,13 @@
         <v>5</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="D5" s="5">
-        <v>18730</v>
+        <v>16050</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
@@ -745,13 +745,13 @@
         <v>5</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D6" s="5">
-        <v>16050</v>
+        <v>18520</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
@@ -759,55 +759,55 @@
         <v>5</v>
       </c>
       <c r="B7" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D7" s="5">
+        <v>9130</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A8" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="B8" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="C8" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="D8" s="8">
+        <v>4420</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A9" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="D9" s="5">
+        <v>24180</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A10" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="B10" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="C7" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="D7" s="5">
-        <v>18520</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A8" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="B8" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="C8" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="D8" s="5">
-        <v>9130</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A9" s="6" t="s">
-        <v>5</v>
-      </c>
-      <c r="B9" s="7" t="s">
-        <v>14</v>
-      </c>
-      <c r="C9" s="7" t="s">
-        <v>15</v>
-      </c>
-      <c r="D9" s="8">
-        <v>4420</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A10" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="B10" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="C10" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="D10" s="5">
-        <v>24180</v>
+      <c r="C10" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="D10" s="8">
+        <v>17540</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
@@ -821,21 +821,21 @@
         <v>17</v>
       </c>
       <c r="D11" s="8">
-        <v>17540</v>
+        <v>17730</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A12" s="6" t="s">
-        <v>5</v>
-      </c>
-      <c r="B12" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="C12" s="7" t="s">
-        <v>17</v>
-      </c>
-      <c r="D12" s="8">
-        <v>17730</v>
+      <c r="A12" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="C12" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="D12" s="5">
+        <v>10370</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
@@ -843,13 +843,13 @@
         <v>5</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D13" s="5">
-        <v>10370</v>
+        <v>9590</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
@@ -857,13 +857,13 @@
         <v>5</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D14" s="5">
-        <v>9590</v>
+        <v>11200</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
@@ -871,13 +871,13 @@
         <v>5</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D15" s="5">
-        <v>11200</v>
+        <v>16570</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
@@ -885,13 +885,13 @@
         <v>5</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>9</v>
+        <v>18</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D16" s="5">
-        <v>16570</v>
+        <v>3760</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
@@ -899,13 +899,13 @@
         <v>5</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="D17" s="5">
-        <v>3760</v>
+        <v>8610</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
@@ -916,60 +916,60 @@
         <v>24</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D18" s="5">
-        <v>8610</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A19" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="B19" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="C19" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="D19" s="5">
         <v>8730</v>
       </c>
     </row>
-    <row r="20" ht="24" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A20" s="1" t="s">
+    <row r="19" ht="24" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A19" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="B20" s="1"/>
-      <c r="C20" s="1"/>
-      <c r="D20" s="1"/>
+      <c r="B19" s="1"/>
+      <c r="C19" s="1"/>
+      <c r="D19" s="1"/>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A20" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>4</v>
+      </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A21" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="B21" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="C21" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="D21" s="2" t="s">
-        <v>4</v>
+      <c r="A21" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="B21" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="C21" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="D21" s="5">
+        <v>19070</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22" s="3" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="D22" s="5">
-        <v>19070</v>
+        <v>10690</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
@@ -980,24 +980,24 @@
         <v>32</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D23" s="5">
-        <v>10690</v>
+        <v>11160</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" s="3" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>32</v>
+        <v>24</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D24" s="5">
-        <v>11160</v>
+        <v>9430</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
@@ -1008,46 +1008,46 @@
         <v>24</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="D25" s="5">
-        <v>9430</v>
-      </c>
-    </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A26" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="B26" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="C26" s="4" t="s">
-        <v>36</v>
-      </c>
-      <c r="D26" s="5">
         <v>11250</v>
       </c>
     </row>
-    <row r="27" ht="24" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A27" s="1" t="s">
+    <row r="26" ht="24" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A26" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="B27" s="1"/>
-      <c r="C27" s="1"/>
-      <c r="D27" s="1"/>
+      <c r="B26" s="1"/>
+      <c r="C26" s="1"/>
+      <c r="D26" s="1"/>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A27" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B27" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C27" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="D27" s="2" t="s">
+        <v>4</v>
+      </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A28" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="B28" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="C28" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="D28" s="2" t="s">
-        <v>4</v>
+      <c r="A28" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="B28" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="C28" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="D28" s="5">
+        <v>18470</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.25">
@@ -1055,13 +1055,13 @@
         <v>38</v>
       </c>
       <c r="B29" s="4" t="s">
-        <v>39</v>
+        <v>24</v>
       </c>
       <c r="C29" s="4" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D29" s="5">
-        <v>18470</v>
+        <v>12480</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.25">
@@ -1069,13 +1069,13 @@
         <v>38</v>
       </c>
       <c r="B30" s="4" t="s">
-        <v>24</v>
+        <v>42</v>
       </c>
       <c r="C30" s="4" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="D30" s="5">
-        <v>12480</v>
+        <v>18910</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.25">
@@ -1083,41 +1083,41 @@
         <v>38</v>
       </c>
       <c r="B31" s="4" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="C31" s="4" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="D31" s="5">
-        <v>18910</v>
+        <v>13800</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A32" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="B32" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="C32" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="D32" s="5">
+        <v>3010</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A33" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="B32" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="C32" s="4" t="s">
-        <v>45</v>
-      </c>
-      <c r="D32" s="5">
-        <v>13800</v>
-      </c>
-    </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A33" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="B33" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="C33" s="4" t="s">
-        <v>48</v>
-      </c>
-      <c r="D33" s="5">
-        <v>3010</v>
+      <c r="B33" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="C33" s="7" t="s">
+        <v>49</v>
+      </c>
+      <c r="D33" s="8">
+        <v>26510</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.25">
@@ -1128,52 +1128,52 @@
         <v>14</v>
       </c>
       <c r="C34" s="7" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="D34" s="8">
-        <v>26510</v>
+        <v>26180</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A35" s="6" t="s">
+      <c r="A35" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="B35" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="C35" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="D35" s="5">
+        <v>2630</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A36" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="B35" s="7" t="s">
+      <c r="B36" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="C35" s="7" t="s">
-        <v>50</v>
-      </c>
-      <c r="D35" s="8">
-        <v>26180</v>
-      </c>
-    </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A36" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="B36" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="C36" s="4" t="s">
-        <v>51</v>
-      </c>
-      <c r="D36" s="5">
-        <v>2630</v>
+      <c r="C36" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="D36" s="8">
+        <v>25250</v>
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A37" s="6" t="s">
+      <c r="A37" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="B37" s="7" t="s">
-        <v>14</v>
-      </c>
-      <c r="C37" s="7" t="s">
-        <v>52</v>
-      </c>
-      <c r="D37" s="8">
-        <v>25250</v>
+      <c r="B37" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="C37" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="D37" s="5">
+        <v>20500</v>
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.25">
@@ -1181,41 +1181,41 @@
         <v>38</v>
       </c>
       <c r="B38" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="C38" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="D38" s="5">
+        <v>18400</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A39" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="B39" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="C39" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="D39" s="8">
+        <v>16800</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A40" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="B40" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="C38" s="4" t="s">
-        <v>53</v>
-      </c>
-      <c r="D38" s="5">
-        <v>20500</v>
-      </c>
-    </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A39" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="B39" s="4" t="s">
-        <v>54</v>
-      </c>
-      <c r="C39" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="D39" s="5">
-        <v>18400</v>
-      </c>
-    </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A40" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="B40" s="7" t="s">
-        <v>14</v>
-      </c>
-      <c r="C40" s="7" t="s">
-        <v>56</v>
-      </c>
-      <c r="D40" s="8">
-        <v>16800</v>
+      <c r="C40" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="D40" s="5">
+        <v>14590</v>
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.25">
@@ -1223,85 +1223,85 @@
         <v>38</v>
       </c>
       <c r="B41" s="4" t="s">
-        <v>24</v>
+        <v>47</v>
       </c>
       <c r="C41" s="4" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D41" s="5">
-        <v>14590</v>
-      </c>
-    </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A42" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="B42" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="C42" s="4" t="s">
-        <v>58</v>
-      </c>
-      <c r="D42" s="5">
         <v>2960</v>
       </c>
     </row>
-    <row r="43" ht="24" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A43" s="1" t="s">
+    <row r="42" ht="24" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A42" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="B43" s="1"/>
-      <c r="C43" s="1"/>
-      <c r="D43" s="1"/>
+      <c r="B42" s="1"/>
+      <c r="C42" s="1"/>
+      <c r="D42" s="1"/>
+    </row>
+    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A43" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B43" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C43" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="D43" s="2" t="s">
+        <v>4</v>
+      </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A44" s="2" t="s">
+      <c r="A44" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="B44" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="C44" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="D44" s="5">
+        <v>11000</v>
+      </c>
+    </row>
+    <row r="45" ht="24" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A45" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="B45" s="1"/>
+      <c r="C45" s="1"/>
+      <c r="D45" s="1"/>
+    </row>
+    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A46" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B44" s="2" t="s">
+      <c r="B46" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="C44" s="2" t="s">
+      <c r="C46" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="D44" s="2" t="s">
+      <c r="D46" s="2" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A45" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="B45" s="4" t="s">
-        <v>61</v>
-      </c>
-      <c r="C45" s="4" t="s">
-        <v>62</v>
-      </c>
-      <c r="D45" s="5">
-        <v>11000</v>
-      </c>
-    </row>
-    <row r="46" ht="24" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A46" s="1" t="s">
-        <v>63</v>
-      </c>
-      <c r="B46" s="1"/>
-      <c r="C46" s="1"/>
-      <c r="D46" s="1"/>
-    </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A47" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="B47" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="C47" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="D47" s="2" t="s">
-        <v>4</v>
+      <c r="A47" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="B47" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="C47" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="D47" s="5">
+        <v>3400</v>
       </c>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.25">
@@ -1312,10 +1312,10 @@
         <v>65</v>
       </c>
       <c r="C48" s="4" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="D48" s="5">
-        <v>3400</v>
+        <v>24440</v>
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.25">
@@ -1326,10 +1326,10 @@
         <v>65</v>
       </c>
       <c r="C49" s="4" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D49" s="5">
-        <v>24440</v>
+        <v>24340</v>
       </c>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.25">
@@ -1340,10 +1340,10 @@
         <v>65</v>
       </c>
       <c r="C50" s="4" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D50" s="5">
-        <v>24340</v>
+        <v>57600</v>
       </c>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.25">
@@ -1354,10 +1354,10 @@
         <v>65</v>
       </c>
       <c r="C51" s="4" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="D51" s="5">
-        <v>57600</v>
+        <v>18370</v>
       </c>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.25">
@@ -1368,33 +1368,19 @@
         <v>65</v>
       </c>
       <c r="C52" s="4" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="D52" s="5">
-        <v>18370</v>
-      </c>
-    </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A53" s="3" t="s">
-        <v>64</v>
-      </c>
-      <c r="B53" s="4" t="s">
-        <v>65</v>
-      </c>
-      <c r="C53" s="4" t="s">
-        <v>71</v>
-      </c>
-      <c r="D53" s="5">
         <v>17770</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="5">
     <mergeCell ref="A1:D1"/>
-    <mergeCell ref="A20:D20"/>
-    <mergeCell ref="A27:D27"/>
-    <mergeCell ref="A43:D43"/>
-    <mergeCell ref="A46:D46"/>
+    <mergeCell ref="A19:D19"/>
+    <mergeCell ref="A26:D26"/>
+    <mergeCell ref="A42:D42"/>
+    <mergeCell ref="A45:D45"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
Stok listesi güncellendi (2026-09-28 21:43)
</commit_message>
<xml_diff>
--- a/stok-listesi.xlsx
+++ b/stok-listesi.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="151" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="154" uniqueCount="73">
   <si>
     <t>G A L V A N İ Z L İ   Ü R Ü N L E R</t>
   </si>
@@ -47,6 +47,9 @@
   </si>
   <si>
     <t>1004</t>
+  </si>
+  <si>
+    <t>0,65*1410*2400</t>
   </si>
   <si>
     <t>0,65*1410 R</t>
@@ -667,7 +670,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D52"/>
+  <dimension ref="A1:D53"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -751,7 +754,7 @@
         <v>12</v>
       </c>
       <c r="D6" s="5">
-        <v>18520</v>
+        <v>3453</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
@@ -759,55 +762,55 @@
         <v>5</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="C7" s="4" t="s">
         <v>13</v>
       </c>
       <c r="D7" s="5">
+        <v>15067</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A8" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="D8" s="5">
         <v>9130</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A8" s="6" t="s">
-        <v>5</v>
-      </c>
-      <c r="B8" s="7" t="s">
-        <v>14</v>
-      </c>
-      <c r="C8" s="7" t="s">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A9" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="B9" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="D8" s="8">
+      <c r="C9" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="D9" s="8">
         <v>4420</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A9" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="B9" s="4" t="s">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A10" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B10" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="C9" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="D9" s="5">
+      <c r="C10" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="D10" s="5">
         <v>24180</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A10" s="6" t="s">
-        <v>5</v>
-      </c>
-      <c r="B10" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="C10" s="7" t="s">
-        <v>17</v>
-      </c>
-      <c r="D10" s="8">
-        <v>17540</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
@@ -818,24 +821,24 @@
         <v>11</v>
       </c>
       <c r="C11" s="7" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D11" s="8">
+        <v>17540</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A12" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="B12" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="C12" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="D12" s="8">
         <v>17730</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A12" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="B12" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="C12" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="D12" s="5">
-        <v>10370</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
@@ -843,13 +846,13 @@
         <v>5</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="C13" s="4" t="s">
         <v>20</v>
       </c>
       <c r="D13" s="5">
-        <v>9590</v>
+        <v>10370</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
@@ -857,13 +860,13 @@
         <v>5</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="C14" s="4" t="s">
         <v>21</v>
       </c>
       <c r="D14" s="5">
-        <v>11200</v>
+        <v>9590</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
@@ -871,13 +874,13 @@
         <v>5</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="C15" s="4" t="s">
         <v>22</v>
       </c>
       <c r="D15" s="5">
-        <v>16570</v>
+        <v>11200</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
@@ -885,13 +888,13 @@
         <v>5</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="C16" s="4" t="s">
         <v>23</v>
       </c>
       <c r="D16" s="5">
-        <v>3760</v>
+        <v>16570</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
@@ -899,13 +902,13 @@
         <v>5</v>
       </c>
       <c r="B17" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="C17" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="C17" s="4" t="s">
-        <v>25</v>
-      </c>
       <c r="D17" s="5">
-        <v>8610</v>
+        <v>3760</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
@@ -913,474 +916,488 @@
         <v>5</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C18" s="4" t="s">
         <v>26</v>
       </c>
       <c r="D18" s="5">
+        <v>8610</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A19" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B19" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="C19" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="D19" s="5">
         <v>8730</v>
       </c>
     </row>
-    <row r="19" ht="24" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A19" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="B19" s="1"/>
-      <c r="C19" s="1"/>
-      <c r="D19" s="1"/>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A20" s="2" t="s">
+    <row r="20" ht="24" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A20" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="B20" s="1"/>
+      <c r="C20" s="1"/>
+      <c r="D20" s="1"/>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A21" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B20" s="2" t="s">
+      <c r="B21" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="C20" s="2" t="s">
+      <c r="C21" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="D20" s="2" t="s">
+      <c r="D21" s="2" t="s">
         <v>4</v>
-      </c>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A21" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="B21" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="C21" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="D21" s="5">
-        <v>19070</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="B22" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="C22" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="B22" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="C22" s="4" t="s">
-        <v>33</v>
-      </c>
       <c r="D22" s="5">
-        <v>10690</v>
+        <v>19070</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23" s="3" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B23" s="4" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C23" s="4" t="s">
         <v>34</v>
       </c>
       <c r="D23" s="5">
-        <v>11160</v>
+        <v>10690</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" s="3" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>24</v>
+        <v>33</v>
       </c>
       <c r="C24" s="4" t="s">
         <v>35</v>
       </c>
       <c r="D24" s="5">
-        <v>9430</v>
+        <v>11160</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25" s="3" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C25" s="4" t="s">
         <v>36</v>
       </c>
       <c r="D25" s="5">
+        <v>9430</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A26" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="B26" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="C26" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="D26" s="5">
         <v>11250</v>
       </c>
     </row>
-    <row r="26" ht="24" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A26" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="B26" s="1"/>
-      <c r="C26" s="1"/>
-      <c r="D26" s="1"/>
-    </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A27" s="2" t="s">
+    <row r="27" ht="24" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A27" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="B27" s="1"/>
+      <c r="C27" s="1"/>
+      <c r="D27" s="1"/>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A28" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B27" s="2" t="s">
+      <c r="B28" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="C27" s="2" t="s">
+      <c r="C28" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="D27" s="2" t="s">
+      <c r="D28" s="2" t="s">
         <v>4</v>
-      </c>
-    </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A28" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="B28" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="C28" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="D28" s="5">
-        <v>18470</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A29" s="3" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B29" s="4" t="s">
-        <v>24</v>
+        <v>40</v>
       </c>
       <c r="C29" s="4" t="s">
         <v>41</v>
       </c>
       <c r="D29" s="5">
-        <v>12480</v>
+        <v>18470</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A30" s="3" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B30" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="C30" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="C30" s="4" t="s">
-        <v>43</v>
-      </c>
       <c r="D30" s="5">
-        <v>18910</v>
+        <v>12480</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A31" s="3" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B31" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="C31" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="C31" s="4" t="s">
-        <v>45</v>
-      </c>
       <c r="D31" s="5">
-        <v>13800</v>
+        <v>18910</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A32" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="B32" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="C32" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="B32" s="4" t="s">
+      <c r="D32" s="5">
+        <v>13800</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A33" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="C32" s="4" t="s">
+      <c r="B33" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="D32" s="5">
+      <c r="C33" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="D33" s="5">
         <v>3010</v>
-      </c>
-    </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A33" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="B33" s="7" t="s">
-        <v>14</v>
-      </c>
-      <c r="C33" s="7" t="s">
-        <v>49</v>
-      </c>
-      <c r="D33" s="8">
-        <v>26510</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A34" s="6" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B34" s="7" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C34" s="7" t="s">
         <v>50</v>
       </c>
       <c r="D34" s="8">
+        <v>26510</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A35" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="B35" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="C35" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="D35" s="8">
         <v>26180</v>
       </c>
     </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A35" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="B35" s="4" t="s">
+    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A36" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="C35" s="4" t="s">
-        <v>51</v>
-      </c>
-      <c r="D35" s="5">
+      <c r="B36" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="C36" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="D36" s="5">
         <v>2630</v>
       </c>
     </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A36" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="B36" s="7" t="s">
-        <v>14</v>
-      </c>
-      <c r="C36" s="7" t="s">
-        <v>52</v>
-      </c>
-      <c r="D36" s="8">
+    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A37" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="B37" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="C37" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="D37" s="8">
         <v>25250</v>
-      </c>
-    </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A37" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="B37" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="C37" s="4" t="s">
-        <v>53</v>
-      </c>
-      <c r="D37" s="5">
-        <v>20500</v>
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A38" s="3" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B38" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="C38" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="C38" s="4" t="s">
+      <c r="D38" s="5">
+        <v>20500</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A39" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="B39" s="4" t="s">
         <v>55</v>
       </c>
-      <c r="D38" s="5">
+      <c r="C39" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="D39" s="5">
         <v>18400</v>
       </c>
     </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A39" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="B39" s="7" t="s">
-        <v>14</v>
-      </c>
-      <c r="C39" s="7" t="s">
-        <v>56</v>
-      </c>
-      <c r="D39" s="8">
+    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A40" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="B40" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="C40" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="D40" s="8">
         <v>16800</v>
-      </c>
-    </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A40" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="B40" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="C40" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="D40" s="5">
-        <v>14590</v>
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A41" s="3" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B41" s="4" t="s">
-        <v>47</v>
+        <v>25</v>
       </c>
       <c r="C41" s="4" t="s">
         <v>58</v>
       </c>
       <c r="D41" s="5">
+        <v>14590</v>
+      </c>
+    </row>
+    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A42" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="B42" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="C42" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="D42" s="5">
         <v>2960</v>
       </c>
     </row>
-    <row r="42" ht="24" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A42" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="B42" s="1"/>
-      <c r="C42" s="1"/>
-      <c r="D42" s="1"/>
-    </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A43" s="2" t="s">
+    <row r="43" ht="24" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A43" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="B43" s="1"/>
+      <c r="C43" s="1"/>
+      <c r="D43" s="1"/>
+    </row>
+    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A44" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B43" s="2" t="s">
+      <c r="B44" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="C43" s="2" t="s">
+      <c r="C44" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="D43" s="2" t="s">
+      <c r="D44" s="2" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A44" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="B44" s="4" t="s">
+    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A45" s="3" t="s">
         <v>61</v>
       </c>
-      <c r="C44" s="4" t="s">
+      <c r="B45" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="D44" s="5">
+      <c r="C45" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="D45" s="5">
         <v>11000</v>
       </c>
     </row>
-    <row r="45" ht="24" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A45" s="1" t="s">
-        <v>63</v>
-      </c>
-      <c r="B45" s="1"/>
-      <c r="C45" s="1"/>
-      <c r="D45" s="1"/>
-    </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A46" s="2" t="s">
+    <row r="46" ht="24" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A46" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="B46" s="1"/>
+      <c r="C46" s="1"/>
+      <c r="D46" s="1"/>
+    </row>
+    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A47" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B46" s="2" t="s">
+      <c r="B47" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="C46" s="2" t="s">
+      <c r="C47" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="D46" s="2" t="s">
+      <c r="D47" s="2" t="s">
         <v>4</v>
-      </c>
-    </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A47" s="3" t="s">
-        <v>64</v>
-      </c>
-      <c r="B47" s="4" t="s">
-        <v>65</v>
-      </c>
-      <c r="C47" s="4" t="s">
-        <v>66</v>
-      </c>
-      <c r="D47" s="5">
-        <v>3400</v>
       </c>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A48" s="3" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B48" s="4" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C48" s="4" t="s">
         <v>67</v>
       </c>
       <c r="D48" s="5">
-        <v>24440</v>
+        <v>3400</v>
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A49" s="3" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B49" s="4" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C49" s="4" t="s">
         <v>68</v>
       </c>
       <c r="D49" s="5">
-        <v>24340</v>
+        <v>24440</v>
       </c>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A50" s="3" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B50" s="4" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C50" s="4" t="s">
         <v>69</v>
       </c>
       <c r="D50" s="5">
-        <v>57600</v>
+        <v>24340</v>
       </c>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A51" s="3" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B51" s="4" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C51" s="4" t="s">
         <v>70</v>
       </c>
       <c r="D51" s="5">
-        <v>18370</v>
+        <v>57600</v>
       </c>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A52" s="3" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B52" s="4" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C52" s="4" t="s">
         <v>71</v>
       </c>
       <c r="D52" s="5">
+        <v>18370</v>
+      </c>
+    </row>
+    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A53" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="B53" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="C53" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="D53" s="5">
         <v>17770</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="5">
     <mergeCell ref="A1:D1"/>
-    <mergeCell ref="A19:D19"/>
-    <mergeCell ref="A26:D26"/>
-    <mergeCell ref="A42:D42"/>
-    <mergeCell ref="A45:D45"/>
+    <mergeCell ref="A20:D20"/>
+    <mergeCell ref="A27:D27"/>
+    <mergeCell ref="A43:D43"/>
+    <mergeCell ref="A46:D46"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
Stok listesi güncellendi (2026-10-01 00:23)
</commit_message>
<xml_diff>
--- a/stok-listesi.xlsx
+++ b/stok-listesi.xlsx
@@ -1124,30 +1124,30 @@
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A34" s="6" t="s">
+      <c r="A34" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="B34" s="7" t="s">
+      <c r="B34" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="C34" s="7" t="s">
+      <c r="C34" s="4" t="s">
         <v>50</v>
       </c>
-      <c r="D34" s="8">
+      <c r="D34" s="5">
         <v>26510</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A35" s="6" t="s">
+      <c r="A35" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="B35" s="7" t="s">
+      <c r="B35" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="C35" s="7" t="s">
+      <c r="C35" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="D35" s="8">
+      <c r="D35" s="5">
         <v>26180</v>
       </c>
     </row>
@@ -1166,16 +1166,16 @@
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A37" s="6" t="s">
+      <c r="A37" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="B37" s="7" t="s">
+      <c r="B37" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="C37" s="7" t="s">
+      <c r="C37" s="4" t="s">
         <v>53</v>
       </c>
-      <c r="D37" s="8">
+      <c r="D37" s="5">
         <v>25250</v>
       </c>
     </row>
@@ -1208,16 +1208,16 @@
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A40" s="6" t="s">
+      <c r="A40" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="B40" s="7" t="s">
+      <c r="B40" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="C40" s="7" t="s">
+      <c r="C40" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="D40" s="8">
+      <c r="D40" s="5">
         <v>16800</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Stok listesi güncellendi (2026-10-01 10:18)
</commit_message>
<xml_diff>
--- a/stok-listesi.xlsx
+++ b/stok-listesi.xlsx
@@ -786,16 +786,16 @@
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A9" s="6" t="s">
-        <v>5</v>
-      </c>
-      <c r="B9" s="7" t="s">
+      <c r="A9" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B9" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="C9" s="7" t="s">
+      <c r="C9" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="D9" s="8">
+      <c r="D9" s="5">
         <v>4420</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Stok listesi güncellendi (2026-10-01 10:19)
</commit_message>
<xml_diff>
--- a/stok-listesi.xlsx
+++ b/stok-listesi.xlsx
@@ -236,7 +236,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -251,13 +251,6 @@
     </font>
     <font>
       <b/>
-    </font>
-    <font>
-      <b/>
-      <color rgb="FFFF0000"/>
-    </font>
-    <font>
-      <color rgb="FFFF0000"/>
     </font>
   </fonts>
   <fills count="4">
@@ -305,7 +298,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -320,15 +313,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -814,30 +798,30 @@
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A11" s="6" t="s">
-        <v>5</v>
-      </c>
-      <c r="B11" s="7" t="s">
+      <c r="A11" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B11" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="C11" s="7" t="s">
+      <c r="C11" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="D11" s="8">
+      <c r="D11" s="5">
         <v>17540</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A12" s="6" t="s">
-        <v>5</v>
-      </c>
-      <c r="B12" s="7" t="s">
+      <c r="A12" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B12" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="C12" s="7" t="s">
+      <c r="C12" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="D12" s="8">
+      <c r="D12" s="5">
         <v>17730</v>
       </c>
     </row>

</xml_diff>